<commit_message>
API Test completed with POSTMAN , defect report updated
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Test Plan/Automation Exercise Requirements Traceability Matrix.xlsx
+++ b/Automation Exercise Project/Test Plan/Automation Exercise Requirements Traceability Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgmcm\OneDrive\Desktop\QA Portfolio\Qa-Portfolio\Automation Exercise Project\Test Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E684311F-19D6-43DF-8B80-5B32975CC4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DDFB38-743B-497B-8492-E6442DAD1736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5950" yWindow="3530" windowWidth="28800" windowHeight="15370" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6510" yWindow="3730" windowWidth="28800" windowHeight="15370" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="432">
   <si>
     <t>Automation Exercise | Requirements Traceability Matrix</t>
   </si>
@@ -1557,12 +1557,54 @@
   <si>
     <t xml:space="preserve"> </t>
   </si>
+  <si>
+    <t>API-PRODUCT-001</t>
+  </si>
+  <si>
+    <t>API-BRAND-001</t>
+  </si>
+  <si>
+    <t>API-SEARCH-001</t>
+  </si>
+  <si>
+    <t>API-SEARCH-002</t>
+  </si>
+  <si>
+    <t>API-AUTH-001</t>
+  </si>
+  <si>
+    <t>API-AUTH-002</t>
+  </si>
+  <si>
+    <t>API-PRODUCT-002</t>
+  </si>
+  <si>
+    <t>API-BRAND-002</t>
+  </si>
+  <si>
+    <t>API-AUTH-004</t>
+  </si>
+  <si>
+    <t>API-AUTH-003</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-001</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-002</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-003</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-004</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1620,6 +1662,10 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -1992,6 +2038,43 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2067,43 +2150,6 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2111,13 +2157,69 @@
   </cellStyles>
   <dxfs count="17">
     <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2256,69 +2358,13 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2393,13 +2439,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2573,17 +2619,17 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="OfficialApiScenarios" displayName="OfficialApiScenarios" ref="A4:H18" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="OfficialApiScenarios" displayName="OfficialApiScenarios" ref="A4:H18" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
   <autoFilter ref="A4:H18" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Source API ID" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Exact Scenario Title" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="API URL" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Request Method" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Exact Request Parameter(s)" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Response Code" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Response Type" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Exact Expected Response" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Source API ID" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Exact Scenario Title" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="API URL" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Request Method" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Exact Request Parameter(s)" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Response Code" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Response Type" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Exact Expected Response" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2748,341 +2794,341 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="36" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
     </row>
     <row r="2" spans="1:14" ht="24" customHeight="1">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="41" t="s">
         <v>282</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="E4" s="29" t="s">
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="E4" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="I4" s="29" t="s">
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="I4" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
-      <c r="M4" s="29" t="s">
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="M4" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="29"/>
+      <c r="N4" s="42"/>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="30">
+      <c r="A5" s="43">
         <f>COUNTA(RTM!A8:A107)</f>
         <v>44</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="32"/>
-      <c r="E5" s="30">
+      <c r="B5" s="44"/>
+      <c r="C5" s="45"/>
+      <c r="E5" s="43">
         <f>COUNTIF(RTM!G8:G107,"Fully Covered")</f>
-        <v>13</v>
-      </c>
-      <c r="F5" s="31"/>
-      <c r="G5" s="32"/>
-      <c r="I5" s="30">
+        <v>27</v>
+      </c>
+      <c r="F5" s="44"/>
+      <c r="G5" s="45"/>
+      <c r="I5" s="43">
         <f>COUNTIF(RTM!G8:G107,"Partially Covered")</f>
         <v>1</v>
       </c>
-      <c r="J5" s="31"/>
-      <c r="K5" s="32"/>
-      <c r="M5" s="30">
+      <c r="J5" s="44"/>
+      <c r="K5" s="45"/>
+      <c r="M5" s="43">
         <f>COUNTIF(RTM!G8:G107,"Not Covered")</f>
-        <v>30</v>
-      </c>
-      <c r="N5" s="32"/>
+        <v>16</v>
+      </c>
+      <c r="N5" s="45"/>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="33"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="35"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="35"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="35"/>
-      <c r="M6" s="33"/>
-      <c r="N6" s="35"/>
+      <c r="A6" s="46"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="48"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="48"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="48"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="48"/>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="17" t="s">
         <v>283</v>
       </c>
-      <c r="D8" s="44" t="s">
+      <c r="D8" s="17" t="s">
         <v>284</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="17" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="45" t="s">
+      <c r="A9" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="45">
+      <c r="B9" s="18">
         <f>COUNTIF(RTM!G8:G107,"Fully Covered")</f>
-        <v>13</v>
-      </c>
-      <c r="C9" s="45">
+        <v>27</v>
+      </c>
+      <c r="C9" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site Scenario",RTM!G8:G107,"Fully Covered")</f>
         <v>9</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site API Scenario",RTM!G8:G107,"Fully Covered")</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="45">
+        <v>14</v>
+      </c>
+      <c r="E9" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Tester-Derived",RTM!G8:G107,"Fully Covered")</f>
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:14">
-      <c r="A10" s="45" t="s">
+      <c r="A10" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="45">
+      <c r="B10" s="18">
         <f>COUNTIF(RTM!G8:G107,"Partially Covered")</f>
         <v>1</v>
       </c>
-      <c r="C10" s="45">
+      <c r="C10" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site Scenario",RTM!G8:G107,"Partially Covered")</f>
         <v>1</v>
       </c>
-      <c r="D10" s="45">
+      <c r="D10" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site API Scenario",RTM!G8:G107,"Partially Covered")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="45">
+      <c r="E10" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Tester-Derived",RTM!G8:G107,"Partially Covered")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="45">
+      <c r="B11" s="18">
         <f>COUNTIF(RTM!G8:G107,"Not Covered")</f>
-        <v>30</v>
-      </c>
-      <c r="C11" s="45">
+        <v>16</v>
+      </c>
+      <c r="C11" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site Scenario",RTM!G8:G107,"Not Covered")</f>
         <v>16</v>
       </c>
-      <c r="D11" s="45">
+      <c r="D11" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site API Scenario",RTM!G8:G107,"Not Covered")</f>
-        <v>14</v>
-      </c>
-      <c r="E11" s="45">
+        <v>0</v>
+      </c>
+      <c r="E11" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Tester-Derived",RTM!G8:G107,"Not Covered")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:14">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="46" t="s">
+      <c r="C14" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="19" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="37.5">
-      <c r="A15" s="47" t="s">
+      <c r="A15" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="47">
+      <c r="B15" s="20">
         <f>COUNTIF(RTM!K8:K107,"Pass")</f>
         <v>11</v>
       </c>
-      <c r="C15" s="47">
+      <c r="C15" s="20">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="D15" s="47" t="s">
+      <c r="D15" s="20" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="37.5">
-      <c r="A16" s="47" t="s">
+      <c r="A16" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="47">
+      <c r="B16" s="20">
         <f>COUNTIF(RTM!K8:K107,"Fail")</f>
         <v>3</v>
       </c>
-      <c r="C16" s="47">
+      <c r="C16" s="20">
         <f>COUNTIF(RTM!K8:K107,"Fail")</f>
         <v>3</v>
       </c>
-      <c r="D16" s="47" t="s">
+      <c r="D16" s="20" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="25">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="47">
+      <c r="B17" s="20">
         <f>COUNTIF(RTM!K8:K107,"Not Run")</f>
         <v>30</v>
       </c>
-      <c r="C17" s="47">
+      <c r="C17" s="20">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="D17" s="47" t="s">
+      <c r="D17" s="20" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="15.5">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
     </row>
     <row r="21" spans="1:14" ht="30" customHeight="1">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="31" t="s">
         <v>285</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="20"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="32"/>
+      <c r="N21" s="33"/>
     </row>
     <row r="22" spans="1:14" ht="30" customHeight="1">
-      <c r="A22" s="21"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="23"/>
+      <c r="A22" s="34"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35"/>
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="35"/>
+      <c r="K22" s="35"/>
+      <c r="L22" s="35"/>
+      <c r="M22" s="35"/>
+      <c r="N22" s="36"/>
     </row>
     <row r="23" spans="1:14" ht="30" customHeight="1">
-      <c r="A23" s="21"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="23"/>
+      <c r="A23" s="34"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="35"/>
+      <c r="K23" s="35"/>
+      <c r="L23" s="35"/>
+      <c r="M23" s="35"/>
+      <c r="N23" s="36"/>
     </row>
     <row r="24" spans="1:14" ht="30" customHeight="1">
-      <c r="A24" s="21"/>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-      <c r="N24" s="23"/>
+      <c r="A24" s="34"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="35"/>
+      <c r="K24" s="35"/>
+      <c r="L24" s="35"/>
+      <c r="M24" s="35"/>
+      <c r="N24" s="36"/>
     </row>
     <row r="25" spans="1:14" ht="30" customHeight="1">
-      <c r="A25" s="24"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="J25" s="25"/>
-      <c r="K25" s="25"/>
-      <c r="L25" s="25"/>
-      <c r="M25" s="25"/>
-      <c r="N25" s="26"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38"/>
+      <c r="K25" s="38"/>
+      <c r="L25" s="38"/>
+      <c r="M25" s="38"/>
+      <c r="N25" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3123,70 +3169,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="36" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="37"/>
-      <c r="K4" s="37"/>
-      <c r="L4" s="37"/>
-      <c r="M4" s="38"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+      <c r="J4" s="50"/>
+      <c r="K4" s="50"/>
+      <c r="L4" s="50"/>
+      <c r="M4" s="51"/>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="39"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="41"/>
+      <c r="A5" s="52"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="54"/>
     </row>
     <row r="7" spans="1:13" ht="42" customHeight="1">
       <c r="A7" s="1" t="s">
@@ -4374,570 +4420,598 @@
       </c>
     </row>
     <row r="38" spans="1:15" ht="57" customHeight="1">
-      <c r="A38" s="50" t="s">
+      <c r="A38" s="23" t="s">
         <v>286</v>
       </c>
-      <c r="B38" s="50" t="s">
+      <c r="B38" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C38" s="50" t="s">
+      <c r="C38" s="23" t="s">
         <v>288</v>
       </c>
-      <c r="D38" s="50" t="s">
+      <c r="D38" s="23" t="s">
         <v>289</v>
       </c>
-      <c r="E38" s="50" t="s">
+      <c r="E38" s="23" t="s">
         <v>290</v>
       </c>
-      <c r="F38" s="51"/>
-      <c r="G38" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H38" s="52" t="s">
+      <c r="F38" s="23" t="s">
+        <v>418</v>
+      </c>
+      <c r="G38" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H38" s="25" t="s">
         <v>414</v>
       </c>
-      <c r="I38" s="50" t="s">
+      <c r="I38" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J38" s="50" t="s">
+      <c r="J38" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K38" s="50" t="s">
+      <c r="K38" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L38" s="51"/>
-      <c r="M38" s="50" t="s">
+      <c r="L38" s="24"/>
+      <c r="M38" s="23" t="s">
         <v>292</v>
       </c>
-      <c r="N38" s="53"/>
-      <c r="O38" s="53"/>
+      <c r="N38" s="26"/>
+      <c r="O38" s="26"/>
     </row>
     <row r="39" spans="1:15" ht="57" customHeight="1">
-      <c r="A39" s="50" t="s">
+      <c r="A39" s="23" t="s">
         <v>293</v>
       </c>
-      <c r="B39" s="50" t="s">
+      <c r="B39" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C39" s="50" t="s">
+      <c r="C39" s="23" t="s">
         <v>294</v>
       </c>
-      <c r="D39" s="50" t="s">
+      <c r="D39" s="23" t="s">
         <v>289</v>
       </c>
-      <c r="E39" s="50" t="s">
+      <c r="E39" s="23" t="s">
         <v>295</v>
       </c>
-      <c r="F39" s="51"/>
-      <c r="G39" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H39" s="51" t="s">
+      <c r="F39" s="23" t="s">
+        <v>424</v>
+      </c>
+      <c r="G39" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H39" s="24" t="s">
         <v>296</v>
       </c>
-      <c r="I39" s="50" t="s">
+      <c r="I39" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="J39" s="50" t="s">
+      <c r="J39" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="K39" s="50" t="s">
+      <c r="K39" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L39" s="51"/>
-      <c r="M39" s="50" t="s">
+      <c r="L39" s="24"/>
+      <c r="M39" s="23" t="s">
         <v>298</v>
       </c>
-      <c r="N39" s="53"/>
-      <c r="O39" s="53"/>
+      <c r="N39" s="26"/>
+      <c r="O39" s="26"/>
     </row>
     <row r="40" spans="1:15" ht="57" customHeight="1">
-      <c r="A40" s="50" t="s">
+      <c r="A40" s="23" t="s">
         <v>299</v>
       </c>
-      <c r="B40" s="50" t="s">
+      <c r="B40" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C40" s="50" t="s">
+      <c r="C40" s="23" t="s">
         <v>300</v>
       </c>
-      <c r="D40" s="50" t="s">
+      <c r="D40" s="23" t="s">
         <v>301</v>
       </c>
-      <c r="E40" s="50" t="s">
+      <c r="E40" s="23" t="s">
         <v>302</v>
       </c>
-      <c r="F40" s="51"/>
-      <c r="G40" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H40" s="52" t="s">
+      <c r="F40" s="23" t="s">
+        <v>419</v>
+      </c>
+      <c r="G40" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H40" s="25" t="s">
         <v>414</v>
       </c>
-      <c r="I40" s="50" t="s">
+      <c r="I40" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J40" s="50" t="s">
+      <c r="J40" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K40" s="50" t="s">
+      <c r="K40" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L40" s="51"/>
-      <c r="M40" s="50" t="s">
+      <c r="L40" s="24"/>
+      <c r="M40" s="23" t="s">
         <v>303</v>
       </c>
-      <c r="N40" s="53"/>
-      <c r="O40" s="53"/>
+      <c r="N40" s="26"/>
+      <c r="O40" s="26"/>
     </row>
     <row r="41" spans="1:15" ht="57" customHeight="1">
-      <c r="A41" s="50" t="s">
+      <c r="A41" s="23" t="s">
         <v>304</v>
       </c>
-      <c r="B41" s="50" t="s">
+      <c r="B41" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C41" s="50" t="s">
+      <c r="C41" s="23" t="s">
         <v>305</v>
       </c>
-      <c r="D41" s="50" t="s">
+      <c r="D41" s="23" t="s">
         <v>301</v>
       </c>
-      <c r="E41" s="50" t="s">
+      <c r="E41" s="23" t="s">
         <v>306</v>
       </c>
-      <c r="F41" s="51"/>
-      <c r="G41" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H41" s="51" t="s">
+      <c r="F41" s="23" t="s">
+        <v>425</v>
+      </c>
+      <c r="G41" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H41" s="24" t="s">
         <v>296</v>
       </c>
-      <c r="I41" s="50" t="s">
+      <c r="I41" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="J41" s="50" t="s">
+      <c r="J41" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="K41" s="50" t="s">
+      <c r="K41" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L41" s="51"/>
-      <c r="M41" s="50" t="s">
+      <c r="L41" s="24"/>
+      <c r="M41" s="23" t="s">
         <v>307</v>
       </c>
-      <c r="N41" s="53"/>
-      <c r="O41" s="53"/>
+      <c r="N41" s="26"/>
+      <c r="O41" s="26"/>
     </row>
     <row r="42" spans="1:15" ht="57" customHeight="1">
-      <c r="A42" s="50" t="s">
+      <c r="A42" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="B42" s="50" t="s">
+      <c r="B42" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C42" s="50" t="s">
+      <c r="C42" s="23" t="s">
         <v>309</v>
       </c>
-      <c r="D42" s="50" t="s">
+      <c r="D42" s="23" t="s">
         <v>310</v>
       </c>
-      <c r="E42" s="50" t="s">
+      <c r="E42" s="23" t="s">
         <v>311</v>
       </c>
-      <c r="F42" s="51"/>
-      <c r="G42" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H42" s="51" t="s">
+      <c r="F42" s="23" t="s">
+        <v>420</v>
+      </c>
+      <c r="G42" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H42" s="24" t="s">
         <v>312</v>
       </c>
-      <c r="I42" s="50" t="s">
+      <c r="I42" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J42" s="50" t="s">
+      <c r="J42" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K42" s="50" t="s">
+      <c r="K42" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L42" s="51"/>
-      <c r="M42" s="50" t="s">
+      <c r="L42" s="24"/>
+      <c r="M42" s="23" t="s">
         <v>313</v>
       </c>
-      <c r="N42" s="53"/>
-      <c r="O42" s="53"/>
+      <c r="N42" s="26"/>
+      <c r="O42" s="26"/>
     </row>
     <row r="43" spans="1:15" ht="57" customHeight="1">
-      <c r="A43" s="50" t="s">
+      <c r="A43" s="23" t="s">
         <v>314</v>
       </c>
-      <c r="B43" s="50" t="s">
+      <c r="B43" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C43" s="50" t="s">
+      <c r="C43" s="23" t="s">
         <v>315</v>
       </c>
-      <c r="D43" s="50" t="s">
+      <c r="D43" s="23" t="s">
         <v>310</v>
       </c>
-      <c r="E43" s="54" t="s">
+      <c r="E43" s="27" t="s">
         <v>411</v>
       </c>
-      <c r="F43" s="51"/>
-      <c r="G43" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H43" s="52" t="s">
+      <c r="F43" s="23" t="s">
+        <v>421</v>
+      </c>
+      <c r="G43" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H43" s="25" t="s">
         <v>413</v>
       </c>
-      <c r="I43" s="50" t="s">
+      <c r="I43" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="J43" s="50" t="s">
+      <c r="J43" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K43" s="50" t="s">
+      <c r="K43" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L43" s="51"/>
-      <c r="M43" s="54" t="s">
+      <c r="L43" s="24"/>
+      <c r="M43" s="27" t="s">
         <v>415</v>
       </c>
-      <c r="N43" s="53"/>
-      <c r="O43" s="53"/>
+      <c r="N43" s="26"/>
+      <c r="O43" s="26"/>
     </row>
     <row r="44" spans="1:15" ht="57" customHeight="1">
-      <c r="A44" s="50" t="s">
+      <c r="A44" s="23" t="s">
         <v>316</v>
       </c>
-      <c r="B44" s="50" t="s">
+      <c r="B44" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C44" s="50" t="s">
+      <c r="C44" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="D44" s="50" t="s">
+      <c r="D44" s="23" t="s">
         <v>318</v>
       </c>
-      <c r="E44" s="50" t="s">
+      <c r="E44" s="23" t="s">
         <v>319</v>
       </c>
-      <c r="F44" s="51"/>
-      <c r="G44" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H44" s="51" t="s">
+      <c r="F44" s="23" t="s">
+        <v>422</v>
+      </c>
+      <c r="G44" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H44" s="24" t="s">
         <v>320</v>
       </c>
-      <c r="I44" s="50" t="s">
+      <c r="I44" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J44" s="50" t="s">
+      <c r="J44" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="K44" s="50" t="s">
+      <c r="K44" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L44" s="51"/>
-      <c r="M44" s="50" t="s">
+      <c r="L44" s="24"/>
+      <c r="M44" s="23" t="s">
         <v>321</v>
       </c>
-      <c r="N44" s="53"/>
-      <c r="O44" s="53"/>
+      <c r="N44" s="26"/>
+      <c r="O44" s="26"/>
     </row>
     <row r="45" spans="1:15" ht="57" customHeight="1">
-      <c r="A45" s="50" t="s">
+      <c r="A45" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="B45" s="50" t="s">
+      <c r="B45" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C45" s="50" t="s">
+      <c r="C45" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="D45" s="50" t="s">
+      <c r="D45" s="23" t="s">
         <v>318</v>
       </c>
-      <c r="E45" s="50" t="s">
+      <c r="E45" s="23" t="s">
         <v>324</v>
       </c>
-      <c r="F45" s="51"/>
-      <c r="G45" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H45" s="51" t="s">
+      <c r="F45" s="23" t="s">
+        <v>423</v>
+      </c>
+      <c r="G45" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H45" s="24" t="s">
         <v>325</v>
       </c>
-      <c r="I45" s="50" t="s">
+      <c r="I45" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="J45" s="50" t="s">
+      <c r="J45" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K45" s="50" t="s">
+      <c r="K45" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L45" s="51"/>
-      <c r="M45" s="50" t="s">
+      <c r="L45" s="24"/>
+      <c r="M45" s="23" t="s">
         <v>326</v>
       </c>
-      <c r="N45" s="53"/>
-      <c r="O45" s="53"/>
+      <c r="N45" s="26"/>
+      <c r="O45" s="26"/>
     </row>
     <row r="46" spans="1:15" ht="57" customHeight="1">
-      <c r="A46" s="50" t="s">
+      <c r="A46" s="23" t="s">
         <v>327</v>
       </c>
-      <c r="B46" s="50" t="s">
+      <c r="B46" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C46" s="50" t="s">
+      <c r="C46" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="D46" s="50" t="s">
+      <c r="D46" s="23" t="s">
         <v>318</v>
       </c>
-      <c r="E46" s="50" t="s">
+      <c r="E46" s="23" t="s">
         <v>329</v>
       </c>
-      <c r="F46" s="51"/>
-      <c r="G46" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H46" s="52" t="s">
+      <c r="F46" s="23" t="s">
+        <v>427</v>
+      </c>
+      <c r="G46" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H46" s="25" t="s">
         <v>412</v>
       </c>
-      <c r="I46" s="50" t="s">
+      <c r="I46" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="J46" s="50" t="s">
+      <c r="J46" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="K46" s="50" t="s">
+      <c r="K46" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L46" s="51"/>
-      <c r="M46" s="50" t="s">
+      <c r="L46" s="24"/>
+      <c r="M46" s="23" t="s">
         <v>330</v>
       </c>
-      <c r="N46" s="53"/>
-      <c r="O46" s="53"/>
+      <c r="N46" s="26"/>
+      <c r="O46" s="26"/>
     </row>
     <row r="47" spans="1:15" ht="57" customHeight="1">
-      <c r="A47" s="50" t="s">
+      <c r="A47" s="23" t="s">
         <v>331</v>
       </c>
-      <c r="B47" s="50" t="s">
+      <c r="B47" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C47" s="50" t="s">
+      <c r="C47" s="23" t="s">
         <v>332</v>
       </c>
-      <c r="D47" s="50" t="s">
+      <c r="D47" s="23" t="s">
         <v>318</v>
       </c>
-      <c r="E47" s="50" t="s">
+      <c r="E47" s="23" t="s">
         <v>333</v>
       </c>
-      <c r="F47" s="51"/>
-      <c r="G47" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H47" s="51" t="s">
+      <c r="F47" s="23" t="s">
+        <v>426</v>
+      </c>
+      <c r="G47" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H47" s="24" t="s">
         <v>334</v>
       </c>
-      <c r="I47" s="50" t="s">
+      <c r="I47" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="J47" s="50" t="s">
+      <c r="J47" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K47" s="50" t="s">
+      <c r="K47" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L47" s="51"/>
-      <c r="M47" s="50" t="s">
+      <c r="L47" s="24"/>
+      <c r="M47" s="23" t="s">
         <v>335</v>
       </c>
-      <c r="N47" s="53"/>
-      <c r="O47" s="53"/>
+      <c r="N47" s="26"/>
+      <c r="O47" s="26"/>
     </row>
     <row r="48" spans="1:15" ht="57" customHeight="1">
-      <c r="A48" s="50" t="s">
+      <c r="A48" s="23" t="s">
         <v>336</v>
       </c>
-      <c r="B48" s="50" t="s">
+      <c r="B48" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C48" s="50" t="s">
+      <c r="C48" s="23" t="s">
         <v>337</v>
       </c>
-      <c r="D48" s="50" t="s">
+      <c r="D48" s="23" t="s">
         <v>338</v>
       </c>
-      <c r="E48" s="50" t="s">
+      <c r="E48" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="F48" s="51"/>
-      <c r="G48" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H48" s="51" t="s">
+      <c r="F48" s="23" t="s">
+        <v>428</v>
+      </c>
+      <c r="G48" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H48" s="24" t="s">
         <v>340</v>
       </c>
-      <c r="I48" s="50" t="s">
+      <c r="I48" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J48" s="50" t="s">
+      <c r="J48" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="K48" s="50" t="s">
+      <c r="K48" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L48" s="51"/>
-      <c r="M48" s="50" t="s">
+      <c r="L48" s="24"/>
+      <c r="M48" s="23" t="s">
         <v>341</v>
       </c>
-      <c r="N48" s="53"/>
-      <c r="O48" s="53"/>
+      <c r="N48" s="26"/>
+      <c r="O48" s="26"/>
     </row>
     <row r="49" spans="1:15" ht="57" customHeight="1">
-      <c r="A49" s="50" t="s">
+      <c r="A49" s="23" t="s">
         <v>342</v>
       </c>
-      <c r="B49" s="50" t="s">
+      <c r="B49" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C49" s="50" t="s">
+      <c r="C49" s="23" t="s">
         <v>343</v>
       </c>
-      <c r="D49" s="50" t="s">
+      <c r="D49" s="23" t="s">
         <v>338</v>
       </c>
-      <c r="E49" s="50" t="s">
+      <c r="E49" s="23" t="s">
         <v>344</v>
       </c>
-      <c r="F49" s="51"/>
-      <c r="G49" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H49" s="51" t="s">
+      <c r="F49" s="23" t="s">
+        <v>429</v>
+      </c>
+      <c r="G49" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H49" s="24" t="s">
         <v>345</v>
       </c>
-      <c r="I49" s="50" t="s">
+      <c r="I49" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J49" s="50" t="s">
+      <c r="J49" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="K49" s="50" t="s">
+      <c r="K49" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L49" s="51"/>
-      <c r="M49" s="50" t="s">
+      <c r="L49" s="24"/>
+      <c r="M49" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="N49" s="53"/>
-      <c r="O49" s="53"/>
+      <c r="N49" s="26"/>
+      <c r="O49" s="26"/>
     </row>
     <row r="50" spans="1:15" ht="57" customHeight="1">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="23" t="s">
         <v>347</v>
       </c>
-      <c r="B50" s="50" t="s">
+      <c r="B50" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C50" s="50" t="s">
+      <c r="C50" s="23" t="s">
         <v>348</v>
       </c>
-      <c r="D50" s="50" t="s">
+      <c r="D50" s="23" t="s">
         <v>338</v>
       </c>
-      <c r="E50" s="50" t="s">
+      <c r="E50" s="23" t="s">
         <v>349</v>
       </c>
-      <c r="F50" s="51"/>
-      <c r="G50" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H50" s="51" t="s">
+      <c r="F50" s="23" t="s">
+        <v>430</v>
+      </c>
+      <c r="G50" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H50" s="24" t="s">
         <v>350</v>
       </c>
-      <c r="I50" s="50" t="s">
+      <c r="I50" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J50" s="50" t="s">
+      <c r="J50" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K50" s="50" t="s">
+      <c r="K50" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L50" s="51"/>
-      <c r="M50" s="50" t="s">
+      <c r="L50" s="24"/>
+      <c r="M50" s="23" t="s">
         <v>351</v>
       </c>
-      <c r="N50" s="53"/>
-      <c r="O50" s="53"/>
+      <c r="N50" s="26"/>
+      <c r="O50" s="26"/>
     </row>
     <row r="51" spans="1:15" ht="57" customHeight="1">
-      <c r="A51" s="50" t="s">
+      <c r="A51" s="23" t="s">
         <v>352</v>
       </c>
-      <c r="B51" s="50" t="s">
+      <c r="B51" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="C51" s="50" t="s">
+      <c r="C51" s="23" t="s">
         <v>353</v>
       </c>
-      <c r="D51" s="50" t="s">
+      <c r="D51" s="23" t="s">
         <v>338</v>
       </c>
-      <c r="E51" s="50" t="s">
+      <c r="E51" s="23" t="s">
         <v>354</v>
       </c>
-      <c r="F51" s="51"/>
-      <c r="G51" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="H51" s="51" t="s">
+      <c r="F51" s="23" t="s">
+        <v>431</v>
+      </c>
+      <c r="G51" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="H51" s="24" t="s">
         <v>355</v>
       </c>
-      <c r="I51" s="50" t="s">
+      <c r="I51" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="J51" s="50" t="s">
+      <c r="J51" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K51" s="50" t="s">
+      <c r="K51" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L51" s="51"/>
-      <c r="M51" s="50" t="s">
+      <c r="L51" s="24"/>
+      <c r="M51" s="23" t="s">
         <v>356</v>
       </c>
-      <c r="N51" s="53"/>
-      <c r="O51" s="53"/>
+      <c r="N51" s="26"/>
+      <c r="O51" s="26"/>
     </row>
     <row r="52" spans="1:15" ht="57" customHeight="1">
-      <c r="F52" s="48"/>
-      <c r="G52" s="48"/>
-      <c r="H52" s="48"/>
-      <c r="I52" s="49"/>
-      <c r="J52" s="49"/>
-      <c r="K52" s="49"/>
-      <c r="L52" s="48"/>
-      <c r="M52" s="48"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="21"/>
+      <c r="H52" s="21"/>
+      <c r="I52" s="22"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="22"/>
+      <c r="L52" s="21"/>
+      <c r="M52" s="21"/>
     </row>
     <row r="53" spans="1:15" ht="57" customHeight="1">
-      <c r="F53" s="48"/>
-      <c r="G53" s="48"/>
-      <c r="H53" s="48"/>
-      <c r="I53" s="48"/>
-      <c r="J53" s="48"/>
-      <c r="K53" s="48"/>
-      <c r="L53" s="48"/>
-      <c r="M53" s="48"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="21"/>
+      <c r="H53" s="21"/>
+      <c r="I53" s="21"/>
+      <c r="J53" s="21"/>
+      <c r="K53" s="21"/>
+      <c r="L53" s="21"/>
+      <c r="M53" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4945,15 +5019,16 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A4:M5"/>
   </mergeCells>
+  <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="G8:G107">
-    <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="Fully Covered"/>
-    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="Partially Covered"/>
-    <cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="Not Covered"/>
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Fully Covered"/>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Partially Covered"/>
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Not Covered"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K8:K107">
-    <cfRule type="containsText" dxfId="13" priority="4" operator="containsText" text="Pass"/>
-    <cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Fail"/>
-    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="Not Run"/>
+    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="Pass"/>
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="Fail"/>
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="Not Run"/>
   </conditionalFormatting>
   <dataValidations count="5">
     <dataValidation type="list" sqref="G8:G107" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -4991,20 +5066,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="40" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
     </row>
     <row r="2" spans="1:4" ht="24" customHeight="1">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="41" t="s">
         <v>226</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
     </row>
     <row r="4" spans="1:4" ht="38" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5412,28 +5487,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="28" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="29" t="s">
         <v>416</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="4" spans="1:8" ht="42" customHeight="1">
       <c r="A4" s="16" t="s">

</xml_diff>

<commit_message>
next batch of Test Cases added from the RTM  to test case repository
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Test Plan/Automation Exercise Requirements Traceability Matrix.xlsx
+++ b/Automation Exercise Project/Test Plan/Automation Exercise Requirements Traceability Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgmcm\OneDrive\Desktop\QA Portfolio\Qa-Portfolio\Automation Exercise Project\Test Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DDFB38-743B-497B-8492-E6442DAD1736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C29A31F-3802-4417-A583-49C4CEE3C621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6510" yWindow="3730" windowWidth="28800" windowHeight="15370" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="436">
   <si>
     <t>Automation Exercise | Requirements Traceability Matrix</t>
   </si>
@@ -53,12 +53,24 @@
     <t>Not Covered</t>
   </si>
   <si>
+    <t>Coverage Status</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>UI Scenarios</t>
+  </si>
+  <si>
+    <t>API Scenarios</t>
+  </si>
+  <si>
+    <t>Tester-Derived</t>
+  </si>
+  <si>
     <t>Execution Status</t>
   </si>
   <si>
-    <t>Count</t>
-  </si>
-  <si>
     <t>Defect-Linked</t>
   </si>
   <si>
@@ -89,9 +101,6 @@
     <t>Requirements Traceability Matrix</t>
   </si>
   <si>
-    <t>Coverage is synchronized with the 17-case test repository and four-defect log. Source scenario wording and exact steps are preserved on the Source Scenarios worksheet.</t>
-  </si>
-  <si>
     <t>Coverage rule: Fully Covered means every material behavior in the requirement is mapped to one or more existing test cases. Partially Covered means some, but not all material behavior is mapped. Not Covered means no existing case verifies the requirement.</t>
   </si>
   <si>
@@ -111,9 +120,6 @@
   </si>
   <si>
     <t>Mapped Test Case ID(s)</t>
-  </si>
-  <si>
-    <t>Coverage Status</t>
   </si>
   <si>
     <t>Coverage Rationale</t>
@@ -268,15 +274,9 @@
     <t>Contact Us Form</t>
   </si>
   <si>
-    <t>No contact-form test exists.</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>Create a contact-form case covering file upload, confirmation dialog, success message, and return to Home.</t>
-  </si>
-  <si>
     <t>REQ-NAV-001</t>
   </si>
   <si>
@@ -289,15 +289,9 @@
     <t>Verify Test Cases Page</t>
   </si>
   <si>
-    <t>No navigation test covers the Test Cases page.</t>
-  </si>
-  <si>
     <t>Low</t>
   </si>
   <si>
-    <t>Create a navigation case for the Test Cases page.</t>
-  </si>
-  <si>
     <t>REQ-PRODUCT-001</t>
   </si>
   <si>
@@ -349,12 +343,6 @@
     <t>Verify Subscription in home page</t>
   </si>
   <si>
-    <t>No homepage subscription test exists.</t>
-  </si>
-  <si>
-    <t>Create homepage subscription coverage.</t>
-  </si>
-  <si>
     <t>REQ-SUB-002</t>
   </si>
   <si>
@@ -364,12 +352,6 @@
     <t>Verify Subscription in Cart page</t>
   </si>
   <si>
-    <t>No cart-page subscription test exists.</t>
-  </si>
-  <si>
-    <t>Create cart-page subscription coverage.</t>
-  </si>
-  <si>
     <t>REQ-CART-001</t>
   </si>
   <si>
@@ -637,9 +619,6 @@
     <t>REQ-EXT-001</t>
   </si>
   <si>
-    <t>Tester-Derived</t>
-  </si>
-  <si>
     <t>CUSTOM-01</t>
   </si>
   <si>
@@ -716,6 +695,281 @@
   </si>
   <si>
     <t>Retain as enhanced account-lifecycle coverage.</t>
+  </si>
+  <si>
+    <t>REQ-API-001</t>
+  </si>
+  <si>
+    <t>Site API Scenario</t>
+  </si>
+  <si>
+    <t>SRC-API-01</t>
+  </si>
+  <si>
+    <t>Product API</t>
+  </si>
+  <si>
+    <t>Get All Products List</t>
+  </si>
+  <si>
+    <t>API-PRODUCT-001</t>
+  </si>
+  <si>
+    <t>Official API scenario is documented, but no portfolio API
+ test has been executed.</t>
+  </si>
+  <si>
+    <t>API — Positive</t>
+  </si>
+  <si>
+    <t>Create API-PRODUCT-001 and verify the product-list response.</t>
+  </si>
+  <si>
+    <t>REQ-API-002</t>
+  </si>
+  <si>
+    <t>SRC-API-02</t>
+  </si>
+  <si>
+    <t>POST To All Products List</t>
+  </si>
+  <si>
+    <t>API-PRODUCT-002</t>
+  </si>
+  <si>
+    <t>Unsupported-method handling has not been tested.</t>
+  </si>
+  <si>
+    <t>API — Negative</t>
+  </si>
+  <si>
+    <t>Create API-PRODUCT-002 and verify the 405 response behavior.</t>
+  </si>
+  <si>
+    <t>REQ-API-003</t>
+  </si>
+  <si>
+    <t>SRC-API-03</t>
+  </si>
+  <si>
+    <t>Brand API</t>
+  </si>
+  <si>
+    <t>Get All Brands List</t>
+  </si>
+  <si>
+    <t>API-BRAND-001</t>
+  </si>
+  <si>
+    <t>Create API-BRAND-001 and verify the brand-list response.</t>
+  </si>
+  <si>
+    <t>REQ-API-004</t>
+  </si>
+  <si>
+    <t>SRC-API-04</t>
+  </si>
+  <si>
+    <t>PUT To All Brands List</t>
+  </si>
+  <si>
+    <t>API-BRAND-002</t>
+  </si>
+  <si>
+    <t>Create API-BRAND-002 and verify the 405 response behavior.</t>
+  </si>
+  <si>
+    <t>REQ-API-005</t>
+  </si>
+  <si>
+    <t>SRC-API-05</t>
+  </si>
+  <si>
+    <t>Search API</t>
+  </si>
+  <si>
+    <t>POST To Search Product</t>
+  </si>
+  <si>
+    <t>API-SEARCH-001</t>
+  </si>
+  <si>
+    <t>Valid product-search API behavior has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-SEARCH-001 using a valid search_product parameter.</t>
+  </si>
+  <si>
+    <t>REQ-API-006</t>
+  </si>
+  <si>
+    <t>SRC-API-06</t>
+  </si>
+  <si>
+    <t>POST To Search Product without search_product 
+parameter</t>
+  </si>
+  <si>
+    <t>API-SEARCH-002</t>
+  </si>
+  <si>
+    <t>Missing-parameter validation for product search has not
+ been tested.</t>
+  </si>
+  <si>
+    <t>Create API-SEARCH-002 without the required search_product 
+parameter.</t>
+  </si>
+  <si>
+    <t>REQ-API-007</t>
+  </si>
+  <si>
+    <t>SRC-API-07</t>
+  </si>
+  <si>
+    <t>Authentication API</t>
+  </si>
+  <si>
+    <t>POST To Verify Login with valid details</t>
+  </si>
+  <si>
+    <t>API-AUTH-001</t>
+  </si>
+  <si>
+    <t>Valid API login verification has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-AUTH-001 using valid test credentials.</t>
+  </si>
+  <si>
+    <t>REQ-API-008</t>
+  </si>
+  <si>
+    <t>SRC-API-08</t>
+  </si>
+  <si>
+    <t>POST To Verify Login without email parameter</t>
+  </si>
+  <si>
+    <t>API-AUTH-002</t>
+  </si>
+  <si>
+    <t>Missing-email validation for API login has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-AUTH-002 with only the password parameter.</t>
+  </si>
+  <si>
+    <t>REQ-API-009</t>
+  </si>
+  <si>
+    <t>SRC-API-09</t>
+  </si>
+  <si>
+    <t>DELETE To Verify Login</t>
+  </si>
+  <si>
+    <t>API-AUTH-003</t>
+  </si>
+  <si>
+    <t>Unsupported DELETE handling for login verification 
+has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-AUTH-003 and verify the 405 response behavior.</t>
+  </si>
+  <si>
+    <t>REQ-API-010</t>
+  </si>
+  <si>
+    <t>SRC-API-10</t>
+  </si>
+  <si>
+    <t>POST To Verify Login with invalid details</t>
+  </si>
+  <si>
+    <t>API-AUTH-004</t>
+  </si>
+  <si>
+    <t>Invalid API login behavior has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-AUTH-004 using invalid test credentials.</t>
+  </si>
+  <si>
+    <t>REQ-API-011</t>
+  </si>
+  <si>
+    <t>SRC-API-11</t>
+  </si>
+  <si>
+    <t>Account API</t>
+  </si>
+  <si>
+    <t>POST To Create/Register User Account</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-001</t>
+  </si>
+  <si>
+    <t>API account creation has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-ACCOUNT-001 using a disposable test account.</t>
+  </si>
+  <si>
+    <t>REQ-API-012</t>
+  </si>
+  <si>
+    <t>SRC-API-12</t>
+  </si>
+  <si>
+    <t>DELETE METHOD To Delete User Account</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-002</t>
+  </si>
+  <si>
+    <t>API account deletion has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-ACCOUNT-002 and delete only a disposable test account.</t>
+  </si>
+  <si>
+    <t>REQ-API-013</t>
+  </si>
+  <si>
+    <t>SRC-API-13</t>
+  </si>
+  <si>
+    <t>PUT METHOD To Update User Account</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-003</t>
+  </si>
+  <si>
+    <t>API account updates have not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-ACCOUNT-003 and verify the updated account values.</t>
+  </si>
+  <si>
+    <t>REQ-API-014</t>
+  </si>
+  <si>
+    <t>SRC-API-14</t>
+  </si>
+  <si>
+    <t>GET user account detail by email</t>
+  </si>
+  <si>
+    <t>API-ACCOUNT-004</t>
+  </si>
+  <si>
+    <t>API account-detail retrieval has not been tested.</t>
+  </si>
+  <si>
+    <t>Create API-ACCOUNT-004 using a dedicated QA account email.</t>
   </si>
   <si>
     <t>Authoritative Source Scenarios</t>
@@ -1142,237 +1396,12 @@
 7. Verify that page is scrolled up and 'Full-Fledged practice website for Automation Engineers' text is visible on screen</t>
   </si>
   <si>
-    <t>Cross-reference of 26 official UI scenarios, 14 official API scenarios, and 4 tester-derived requirements against the current 17 executed manual UI test cases</t>
-  </si>
-  <si>
-    <t>UI Scenarios</t>
-  </si>
-  <si>
-    <t>API Scenarios</t>
-  </si>
-  <si>
-    <t>Current strength: registration, login, account lifecycle, product discovery, and foundational cart behavior are covered by 17 executed UI test cases.
-API scope added: all 14 official Automation Exercise API scenarios are now documented as traceable requirements and preserved verbatim on the Source APIs worksheet.
-Current API gap: no Postman API cases have been executed yet, so all 14 API requirements remain Not Covered.
-Recommended next action: execute API-PRODUCT-001, API-BRAND-001, API-SEARCH-001, and API-SEARCH-002 in Postman; record both the HTTP status and any responseCode returned inside the JSON; then map the results back to this RTM.</t>
-  </si>
-  <si>
-    <t>REQ-API-001</t>
-  </si>
-  <si>
-    <t>Site API Scenario</t>
-  </si>
-  <si>
-    <t>SRC-API-01</t>
-  </si>
-  <si>
-    <t>Product API</t>
-  </si>
-  <si>
-    <t>Get All Products List</t>
-  </si>
-  <si>
-    <t>API — Positive</t>
-  </si>
-  <si>
-    <t>Create API-PRODUCT-001 and verify the product-list response.</t>
-  </si>
-  <si>
-    <t>REQ-API-002</t>
-  </si>
-  <si>
-    <t>SRC-API-02</t>
-  </si>
-  <si>
-    <t>POST To All Products List</t>
-  </si>
-  <si>
-    <t>Unsupported-method handling has not been tested.</t>
-  </si>
-  <si>
-    <t>API — Negative</t>
-  </si>
-  <si>
-    <t>Create API-PRODUCT-002 and verify the 405 response behavior.</t>
-  </si>
-  <si>
-    <t>REQ-API-003</t>
-  </si>
-  <si>
-    <t>SRC-API-03</t>
-  </si>
-  <si>
-    <t>Brand API</t>
-  </si>
-  <si>
-    <t>Get All Brands List</t>
-  </si>
-  <si>
-    <t>Create API-BRAND-001 and verify the brand-list response.</t>
-  </si>
-  <si>
-    <t>REQ-API-004</t>
-  </si>
-  <si>
-    <t>SRC-API-04</t>
-  </si>
-  <si>
-    <t>PUT To All Brands List</t>
-  </si>
-  <si>
-    <t>Create API-BRAND-002 and verify the 405 response behavior.</t>
-  </si>
-  <si>
-    <t>REQ-API-005</t>
-  </si>
-  <si>
-    <t>SRC-API-05</t>
-  </si>
-  <si>
-    <t>Search API</t>
-  </si>
-  <si>
-    <t>POST To Search Product</t>
-  </si>
-  <si>
-    <t>Valid product-search API behavior has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-SEARCH-001 using a valid search_product parameter.</t>
-  </si>
-  <si>
-    <t>REQ-API-006</t>
-  </si>
-  <si>
-    <t>SRC-API-06</t>
-  </si>
-  <si>
-    <t>REQ-API-007</t>
-  </si>
-  <si>
-    <t>SRC-API-07</t>
-  </si>
-  <si>
-    <t>Authentication API</t>
-  </si>
-  <si>
-    <t>POST To Verify Login with valid details</t>
-  </si>
-  <si>
-    <t>Valid API login verification has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-AUTH-001 using valid test credentials.</t>
-  </si>
-  <si>
-    <t>REQ-API-008</t>
-  </si>
-  <si>
-    <t>SRC-API-08</t>
-  </si>
-  <si>
-    <t>POST To Verify Login without email parameter</t>
-  </si>
-  <si>
-    <t>Missing-email validation for API login has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-AUTH-002 with only the password parameter.</t>
-  </si>
-  <si>
-    <t>REQ-API-009</t>
-  </si>
-  <si>
-    <t>SRC-API-09</t>
-  </si>
-  <si>
-    <t>DELETE To Verify Login</t>
-  </si>
-  <si>
-    <t>Create API-AUTH-003 and verify the 405 response behavior.</t>
-  </si>
-  <si>
-    <t>REQ-API-010</t>
-  </si>
-  <si>
-    <t>SRC-API-10</t>
-  </si>
-  <si>
-    <t>POST To Verify Login with invalid details</t>
-  </si>
-  <si>
-    <t>Invalid API login behavior has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-AUTH-004 using invalid test credentials.</t>
-  </si>
-  <si>
-    <t>REQ-API-011</t>
-  </si>
-  <si>
-    <t>SRC-API-11</t>
-  </si>
-  <si>
-    <t>Account API</t>
-  </si>
-  <si>
-    <t>POST To Create/Register User Account</t>
-  </si>
-  <si>
-    <t>API account creation has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-ACCOUNT-001 using a disposable test account.</t>
-  </si>
-  <si>
-    <t>REQ-API-012</t>
-  </si>
-  <si>
-    <t>SRC-API-12</t>
-  </si>
-  <si>
-    <t>DELETE METHOD To Delete User Account</t>
-  </si>
-  <si>
-    <t>API account deletion has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-ACCOUNT-002 and delete only a disposable test account.</t>
-  </si>
-  <si>
-    <t>REQ-API-013</t>
-  </si>
-  <si>
-    <t>SRC-API-13</t>
-  </si>
-  <si>
-    <t>PUT METHOD To Update User Account</t>
-  </si>
-  <si>
-    <t>API account updates have not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-ACCOUNT-003 and verify the updated account values.</t>
-  </si>
-  <si>
-    <t>REQ-API-014</t>
-  </si>
-  <si>
-    <t>SRC-API-14</t>
-  </si>
-  <si>
-    <t>GET user account detail by email</t>
-  </si>
-  <si>
-    <t>API account-detail retrieval has not been tested.</t>
-  </si>
-  <si>
-    <t>Create API-ACCOUNT-004 using a dedicated QA account email.</t>
-  </si>
-  <si>
     <t>Automation Exercise — Official API Source Scenarios</t>
   </si>
   <si>
+    <t>Exact scenario details transcribed from Automation Exercise Web Application</t>
+  </si>
+  <si>
     <t>Source API ID</t>
   </si>
   <si>
@@ -1520,6 +1549,9 @@
     <t>User updated!</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>API 14: GET user account detail by email</t>
   </si>
   <si>
@@ -1532,79 +1564,59 @@
     <t>User Detail</t>
   </si>
   <si>
-    <t>POST To Search Product without search_product 
-parameter</t>
-  </si>
-  <si>
-    <t>Unsupported DELETE handling for login verification 
-has not been tested.</t>
-  </si>
-  <si>
-    <t>Missing-parameter validation for product search has not
- been tested.</t>
-  </si>
-  <si>
-    <t>Official API scenario is documented, but no portfolio API
- test has been executed.</t>
-  </si>
-  <si>
-    <t>Create API-SEARCH-002 without the required search_product 
-parameter.</t>
-  </si>
-  <si>
-    <t>Exact scenario details transcribed from Automation Exercise Web Application</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>API-PRODUCT-001</t>
-  </si>
-  <si>
-    <t>API-BRAND-001</t>
-  </si>
-  <si>
-    <t>API-SEARCH-001</t>
-  </si>
-  <si>
-    <t>API-SEARCH-002</t>
-  </si>
-  <si>
-    <t>API-AUTH-001</t>
-  </si>
-  <si>
-    <t>API-AUTH-002</t>
-  </si>
-  <si>
-    <t>API-PRODUCT-002</t>
-  </si>
-  <si>
-    <t>API-BRAND-002</t>
-  </si>
-  <si>
-    <t>API-AUTH-004</t>
-  </si>
-  <si>
-    <t>API-AUTH-003</t>
-  </si>
-  <si>
-    <t>API-ACCOUNT-001</t>
-  </si>
-  <si>
-    <t>API-ACCOUNT-002</t>
-  </si>
-  <si>
-    <t>API-ACCOUNT-003</t>
-  </si>
-  <si>
-    <t>API-ACCOUNT-004</t>
+    <t>Cross-reference of 26 official UI scenarios, 14 official API scenarios, and 4 tester-derived requirements against the current 21-case manual UI test repository</t>
+  </si>
+  <si>
+    <t>Current strength: registration, login, account lifecycle, product discovery, foundational cart behavior, contact-form submission, Test Cases navigation, and subscription coverage are mapped across 21 manual UI cases.
+Batch 3 execution is complete: AE-CONTACT-001, AE-NAV-001, AE-SUB-001, and AE-SUB-002 all passed with evidence recorded in the test repository.
+The manual repository now contains 18 passed cases, 3 failed cases, and 0 cases remaining Not Run.
+Recommended next action: retain the Batch 3 evidence for regression coverage and continue creating cases for the remaining uncovered checkout, catalog, review, recommendation, and scroll-navigation requirements.</t>
+  </si>
+  <si>
+    <t>Coverage is synchronized with the 21-case manual test repository and current defect log. Source scenario wording and exact steps are preserved on the Source Scenarios worksheet.</t>
+  </si>
+  <si>
+    <t>AE-CONTACT-001</t>
+  </si>
+  <si>
+    <t>No immediate gap. Preserve the sanitized AE-CONTACT-001 screenshot and successful return-to-Home observation for regression evidence.</t>
+  </si>
+  <si>
+    <t>AE-NAV-001</t>
+  </si>
+  <si>
+    <t>No immediate gap. Retain AE-NAV-001 evidence showing both successful navigation and the published Test Cases page content.</t>
+  </si>
+  <si>
+    <t>AE-SUB-001</t>
+  </si>
+  <si>
+    <t>No immediate gap. Retain the sanitized AE-SUB-001 screenshot and reuse a controlled email value during regression testing.</t>
+  </si>
+  <si>
+    <t>AE-SUB-002</t>
+  </si>
+  <si>
+    <t>No immediate gap. Retain AE-SUB-002 evidence confirming both the success message and continued cart-page context.</t>
+  </si>
+  <si>
+    <t>The home-page footer displayed the subscription heading, accepted the sanitized email, and showed the expected success message.</t>
+  </si>
+  <si>
+    <t>The cart-page footer displayed the subscription heading, accepted the sanitized email, showed the expected success message, and remained on the cart page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Navigation to the Test Cases page completed without error and the published scenarios were visible as expected.</t>
+  </si>
+  <si>
+    <t>Text entry, permitted file upload, the confirmation dialog, success messaging, and return to Home all matched the expected result.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1662,10 +1674,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -2069,12 +2077,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2150,12 +2152,18 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF595959"/>
@@ -2220,151 +2228,6 @@
           <bgColor rgb="FFE2F0D9"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2439,20 +2302,20 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>27</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5753-4948-94F8-7D0C6B4BB87D}"/>
+              <c16:uniqueId val="{00000000-9EFE-469B-8359-D8AD469DDEA2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2619,17 +2482,17 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="OfficialApiScenarios" displayName="OfficialApiScenarios" ref="A4:H18" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="OfficialApiScenarios" displayName="OfficialApiScenarios" ref="A4:H18">
   <autoFilter ref="A4:H18" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Source API ID" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Exact Scenario Title" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="API URL" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Request Method" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Exact Request Parameter(s)" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Response Code" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Response Type" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Exact Expected Response" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Source API ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Exact Scenario Title"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="API URL"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Request Method"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Exact Request Parameter(s)"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Response Code"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Response Type"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Exact Expected Response"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2794,115 +2657,115 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="36" customHeight="1">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
     </row>
     <row r="2" spans="1:14" ht="24" customHeight="1">
-      <c r="A2" s="41" t="s">
-        <v>282</v>
-      </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
+      <c r="A2" s="39" t="s">
+        <v>421</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+      <c r="N2" s="39"/>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="E4" s="42" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="E4" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="I4" s="42" t="s">
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="I4" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="M4" s="42" t="s">
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="M4" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="42"/>
+      <c r="N4" s="40"/>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="43">
+      <c r="A5" s="41">
         <f>COUNTA(RTM!A8:A107)</f>
         <v>44</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="45"/>
-      <c r="E5" s="43">
+      <c r="B5" s="42"/>
+      <c r="C5" s="43"/>
+      <c r="E5" s="41">
         <f>COUNTIF(RTM!G8:G107,"Fully Covered")</f>
-        <v>27</v>
-      </c>
-      <c r="F5" s="44"/>
-      <c r="G5" s="45"/>
-      <c r="I5" s="43">
+        <v>31</v>
+      </c>
+      <c r="F5" s="42"/>
+      <c r="G5" s="43"/>
+      <c r="I5" s="41">
         <f>COUNTIF(RTM!G8:G107,"Partially Covered")</f>
         <v>1</v>
       </c>
-      <c r="J5" s="44"/>
-      <c r="K5" s="45"/>
-      <c r="M5" s="43">
+      <c r="J5" s="42"/>
+      <c r="K5" s="43"/>
+      <c r="M5" s="41">
         <f>COUNTIF(RTM!G8:G107,"Not Covered")</f>
-        <v>16</v>
-      </c>
-      <c r="N5" s="45"/>
+        <v>12</v>
+      </c>
+      <c r="N5" s="43"/>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="46"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="48"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="48"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="48"/>
-      <c r="M6" s="46"/>
-      <c r="N6" s="48"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="46"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="46"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="46"/>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="17" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>283</v>
+        <v>7</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>284</v>
+        <v>8</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>198</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -2911,11 +2774,11 @@
       </c>
       <c r="B9" s="18">
         <f>COUNTIF(RTM!G8:G107,"Fully Covered")</f>
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C9" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site Scenario",RTM!G8:G107,"Fully Covered")</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D9" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site API Scenario",RTM!G8:G107,"Fully Covered")</f>
@@ -2953,11 +2816,11 @@
       </c>
       <c r="B11" s="18">
         <f>COUNTIF(RTM!G8:G107,"Not Covered")</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C11" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site Scenario",RTM!G8:G107,"Not Covered")</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D11" s="18">
         <f>COUNTIFS(RTM!B8:B107,"Site API Scenario",RTM!G8:G107,"Not Covered")</f>
@@ -2970,37 +2833,37 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="19" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>6</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="37.5">
       <c r="A15" s="20" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B15" s="20">
         <f>COUNTIF(RTM!K8:K107,"Pass")</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C15" s="20">
         <f>0</f>
         <v>0</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="37.5">
       <c r="A16" s="20" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B16" s="20">
         <f>COUNTIF(RTM!K8:K107,"Fail")</f>
@@ -3011,124 +2874,124 @@
         <v>3</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="25">
       <c r="A17" s="20" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B17" s="20">
         <f>COUNTIF(RTM!K8:K107,"Not Run")</f>
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C17" s="20">
         <f>0</f>
         <v>0</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="15.5">
-      <c r="A20" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="30"/>
-      <c r="L20" s="30"/>
-      <c r="M20" s="30"/>
-      <c r="N20" s="30"/>
+      <c r="A20" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="28"/>
+      <c r="L20" s="28"/>
+      <c r="M20" s="28"/>
+      <c r="N20" s="28"/>
     </row>
     <row r="21" spans="1:14" ht="30" customHeight="1">
-      <c r="A21" s="31" t="s">
-        <v>285</v>
-      </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-      <c r="N21" s="33"/>
+      <c r="A21" s="29" t="s">
+        <v>422</v>
+      </c>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="30"/>
+      <c r="L21" s="30"/>
+      <c r="M21" s="30"/>
+      <c r="N21" s="31"/>
     </row>
     <row r="22" spans="1:14" ht="30" customHeight="1">
-      <c r="A22" s="34"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="35"/>
-      <c r="M22" s="35"/>
-      <c r="N22" s="36"/>
+      <c r="A22" s="32"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="34"/>
     </row>
     <row r="23" spans="1:14" ht="30" customHeight="1">
-      <c r="A23" s="34"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="35"/>
-      <c r="L23" s="35"/>
-      <c r="M23" s="35"/>
-      <c r="N23" s="36"/>
+      <c r="A23" s="32"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+      <c r="J23" s="33"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="33"/>
+      <c r="N23" s="34"/>
     </row>
     <row r="24" spans="1:14" ht="30" customHeight="1">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="35"/>
-      <c r="L24" s="35"/>
-      <c r="M24" s="35"/>
-      <c r="N24" s="36"/>
+      <c r="A24" s="32"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="33"/>
+      <c r="N24" s="34"/>
     </row>
     <row r="25" spans="1:14" ht="30" customHeight="1">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="38"/>
-      <c r="J25" s="38"/>
-      <c r="K25" s="38"/>
-      <c r="L25" s="38"/>
-      <c r="M25" s="38"/>
-      <c r="N25" s="39"/>
+      <c r="A25" s="35"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="36"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3169,344 +3032,346 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="36" customHeight="1">
-      <c r="A1" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
+      <c r="A1" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1">
-      <c r="A2" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
+      <c r="A2" s="39" t="s">
+        <v>423</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50"/>
-      <c r="L4" s="50"/>
-      <c r="M4" s="51"/>
+      <c r="A4" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="49"/>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="52"/>
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="54"/>
+      <c r="A5" s="50"/>
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="51"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="52"/>
     </row>
     <row r="7" spans="1:13" ht="42" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="57" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>3</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L8" s="5"/>
       <c r="M8" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="57" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="57" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="57" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="57" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L12" s="6"/>
       <c r="M12" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="57" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="G13" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>75</v>
+        <v>435</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>13</v>
       </c>
       <c r="L13" s="6"/>
       <c r="M13" s="8" t="s">
-        <v>77</v>
+        <v>425</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="57" customHeight="1">
@@ -3514,7 +3379,7 @@
         <v>78</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>79</v>
@@ -3525,1470 +3390,1476 @@
       <c r="E14" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="6"/>
+      <c r="F14" s="6" t="s">
+        <v>426</v>
+      </c>
       <c r="G14" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H14" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J14" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>13</v>
       </c>
       <c r="L14" s="6"/>
       <c r="M14" s="8" t="s">
-        <v>84</v>
+        <v>427</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="57" customHeight="1">
       <c r="A15" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="F15" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L15" s="6"/>
       <c r="M15" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="57" customHeight="1">
       <c r="A16" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>95</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L16" s="6"/>
       <c r="M16" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="57" customHeight="1">
       <c r="A17" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="E17" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="6" t="s">
+        <v>428</v>
+      </c>
       <c r="G17" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>102</v>
+        <v>432</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K17" s="5" t="s">
         <v>13</v>
       </c>
       <c r="L17" s="6"/>
       <c r="M17" s="8" t="s">
-        <v>103</v>
+        <v>429</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="57" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F18" s="6"/>
+        <v>102</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>430</v>
+      </c>
       <c r="G18" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>107</v>
+        <v>433</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K18" s="5" t="s">
         <v>13</v>
       </c>
       <c r="L18" s="6"/>
       <c r="M18" s="8" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="57" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="57" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="57" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L21" s="6"/>
       <c r="M21" s="8" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="57" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L22" s="6"/>
       <c r="M22" s="8" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="57" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L23" s="6"/>
       <c r="M23" s="8" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="57" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L24" s="6"/>
       <c r="M24" s="8" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="57" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L25" s="6"/>
       <c r="M25" s="8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="57" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D26" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>149</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>155</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L26" s="6"/>
       <c r="M26" s="8" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="57" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L27" s="6"/>
       <c r="M27" s="8" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="57" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L28" s="6"/>
       <c r="M28" s="8" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="57" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L29" s="6"/>
       <c r="M29" s="8" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="57" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L30" s="6"/>
       <c r="M30" s="8" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="57" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L31" s="6"/>
       <c r="M31" s="8" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="57" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L32" s="6"/>
       <c r="M32" s="8" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" spans="1:15" ht="57" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>80</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
         <v>4</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L33" s="6"/>
       <c r="M33" s="8" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:15" ht="57" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>198</v>
+        <v>9</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L34" s="6"/>
       <c r="M34" s="8" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:15" ht="57" customHeight="1">
       <c r="A35" s="4" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>205</v>
-      </c>
       <c r="D35" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L35" s="6"/>
       <c r="M35" s="8" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:15" ht="57" customHeight="1">
       <c r="A36" s="4" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>198</v>
+        <v>9</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>2</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L36" s="6"/>
       <c r="M36" s="8" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:15" ht="57" customHeight="1">
       <c r="A37" s="9" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>198</v>
+        <v>9</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="G37" s="10" t="s">
         <v>2</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="I37" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J37" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K37" s="10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L37" s="13"/>
       <c r="M37" s="12" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="38" spans="1:15" ht="57" customHeight="1">
       <c r="A38" s="23" t="s">
-        <v>286</v>
+        <v>218</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>288</v>
+        <v>220</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>290</v>
+        <v>222</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>418</v>
+        <v>223</v>
       </c>
       <c r="G38" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H38" s="25" t="s">
-        <v>414</v>
+        <v>224</v>
       </c>
       <c r="I38" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J38" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K38" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L38" s="24"/>
       <c r="M38" s="23" t="s">
-        <v>292</v>
+        <v>226</v>
       </c>
       <c r="N38" s="26"/>
       <c r="O38" s="26"/>
     </row>
     <row r="39" spans="1:15" ht="57" customHeight="1">
       <c r="A39" s="23" t="s">
-        <v>293</v>
+        <v>227</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>294</v>
+        <v>228</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>295</v>
+        <v>229</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>424</v>
+        <v>230</v>
       </c>
       <c r="G39" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H39" s="24" t="s">
-        <v>296</v>
+        <v>231</v>
       </c>
       <c r="I39" s="23" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
       <c r="J39" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K39" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L39" s="24"/>
       <c r="M39" s="23" t="s">
-        <v>298</v>
+        <v>233</v>
       </c>
       <c r="N39" s="26"/>
       <c r="O39" s="26"/>
     </row>
     <row r="40" spans="1:15" ht="57" customHeight="1">
       <c r="A40" s="23" t="s">
-        <v>299</v>
+        <v>234</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>300</v>
+        <v>235</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>301</v>
+        <v>236</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>302</v>
+        <v>237</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>419</v>
+        <v>238</v>
       </c>
       <c r="G40" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H40" s="25" t="s">
-        <v>414</v>
+        <v>224</v>
       </c>
       <c r="I40" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J40" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K40" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L40" s="24"/>
       <c r="M40" s="23" t="s">
-        <v>303</v>
+        <v>239</v>
       </c>
       <c r="N40" s="26"/>
       <c r="O40" s="26"/>
     </row>
     <row r="41" spans="1:15" ht="57" customHeight="1">
       <c r="A41" s="23" t="s">
-        <v>304</v>
+        <v>240</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>305</v>
+        <v>241</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>301</v>
+        <v>236</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>306</v>
+        <v>242</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>425</v>
+        <v>243</v>
       </c>
       <c r="G41" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H41" s="24" t="s">
-        <v>296</v>
+        <v>231</v>
       </c>
       <c r="I41" s="23" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
       <c r="J41" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K41" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L41" s="24"/>
       <c r="M41" s="23" t="s">
-        <v>307</v>
+        <v>244</v>
       </c>
       <c r="N41" s="26"/>
       <c r="O41" s="26"/>
     </row>
     <row r="42" spans="1:15" ht="57" customHeight="1">
       <c r="A42" s="23" t="s">
-        <v>308</v>
+        <v>245</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>309</v>
+        <v>246</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>310</v>
+        <v>247</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>311</v>
+        <v>248</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>420</v>
+        <v>249</v>
       </c>
       <c r="G42" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H42" s="24" t="s">
-        <v>312</v>
+        <v>250</v>
       </c>
       <c r="I42" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J42" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K42" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L42" s="24"/>
       <c r="M42" s="23" t="s">
-        <v>313</v>
+        <v>251</v>
       </c>
       <c r="N42" s="26"/>
       <c r="O42" s="26"/>
     </row>
     <row r="43" spans="1:15" ht="57" customHeight="1">
       <c r="A43" s="23" t="s">
-        <v>314</v>
+        <v>252</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>315</v>
+        <v>253</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>310</v>
+        <v>247</v>
       </c>
       <c r="E43" s="27" t="s">
-        <v>411</v>
+        <v>254</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>421</v>
+        <v>255</v>
       </c>
       <c r="G43" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H43" s="25" t="s">
-        <v>413</v>
+        <v>256</v>
       </c>
       <c r="I43" s="23" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
       <c r="J43" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K43" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L43" s="24"/>
       <c r="M43" s="27" t="s">
-        <v>415</v>
+        <v>257</v>
       </c>
       <c r="N43" s="26"/>
       <c r="O43" s="26"/>
     </row>
     <row r="44" spans="1:15" ht="57" customHeight="1">
       <c r="A44" s="23" t="s">
-        <v>316</v>
+        <v>258</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>317</v>
+        <v>259</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>318</v>
+        <v>260</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>319</v>
+        <v>261</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>422</v>
+        <v>262</v>
       </c>
       <c r="G44" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H44" s="24" t="s">
-        <v>320</v>
+        <v>263</v>
       </c>
       <c r="I44" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J44" s="23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K44" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L44" s="24"/>
       <c r="M44" s="23" t="s">
-        <v>321</v>
+        <v>264</v>
       </c>
       <c r="N44" s="26"/>
       <c r="O44" s="26"/>
     </row>
     <row r="45" spans="1:15" ht="57" customHeight="1">
       <c r="A45" s="23" t="s">
-        <v>322</v>
+        <v>265</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>323</v>
+        <v>266</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>318</v>
+        <v>260</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>324</v>
+        <v>267</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>423</v>
+        <v>268</v>
       </c>
       <c r="G45" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H45" s="24" t="s">
-        <v>325</v>
+        <v>269</v>
       </c>
       <c r="I45" s="23" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
       <c r="J45" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K45" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L45" s="24"/>
       <c r="M45" s="23" t="s">
-        <v>326</v>
+        <v>270</v>
       </c>
       <c r="N45" s="26"/>
       <c r="O45" s="26"/>
     </row>
     <row r="46" spans="1:15" ht="57" customHeight="1">
       <c r="A46" s="23" t="s">
-        <v>327</v>
+        <v>271</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>328</v>
+        <v>272</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>318</v>
+        <v>260</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>329</v>
+        <v>273</v>
       </c>
       <c r="F46" s="23" t="s">
-        <v>427</v>
+        <v>274</v>
       </c>
       <c r="G46" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H46" s="25" t="s">
-        <v>412</v>
+        <v>275</v>
       </c>
       <c r="I46" s="23" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
       <c r="J46" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K46" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L46" s="24"/>
       <c r="M46" s="23" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="N46" s="26"/>
       <c r="O46" s="26"/>
     </row>
     <row r="47" spans="1:15" ht="57" customHeight="1">
       <c r="A47" s="23" t="s">
-        <v>331</v>
+        <v>277</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>332</v>
+        <v>278</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>318</v>
+        <v>260</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>333</v>
+        <v>279</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>426</v>
+        <v>280</v>
       </c>
       <c r="G47" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H47" s="24" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="I47" s="23" t="s">
-        <v>297</v>
+        <v>232</v>
       </c>
       <c r="J47" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K47" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L47" s="24"/>
       <c r="M47" s="23" t="s">
-        <v>335</v>
+        <v>282</v>
       </c>
       <c r="N47" s="26"/>
       <c r="O47" s="26"/>
     </row>
     <row r="48" spans="1:15" ht="57" customHeight="1">
       <c r="A48" s="23" t="s">
-        <v>336</v>
+        <v>283</v>
       </c>
       <c r="B48" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="C48" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="D48" s="23" t="s">
+        <v>285</v>
+      </c>
+      <c r="E48" s="23" t="s">
+        <v>286</v>
+      </c>
+      <c r="F48" s="23" t="s">
         <v>287</v>
-      </c>
-      <c r="C48" s="23" t="s">
-        <v>337</v>
-      </c>
-      <c r="D48" s="23" t="s">
-        <v>338</v>
-      </c>
-      <c r="E48" s="23" t="s">
-        <v>339</v>
-      </c>
-      <c r="F48" s="23" t="s">
-        <v>428</v>
       </c>
       <c r="G48" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H48" s="24" t="s">
-        <v>340</v>
+        <v>288</v>
       </c>
       <c r="I48" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J48" s="23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K48" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L48" s="24"/>
       <c r="M48" s="23" t="s">
-        <v>341</v>
+        <v>289</v>
       </c>
       <c r="N48" s="26"/>
       <c r="O48" s="26"/>
     </row>
     <row r="49" spans="1:15" ht="57" customHeight="1">
       <c r="A49" s="23" t="s">
-        <v>342</v>
+        <v>290</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>343</v>
+        <v>291</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>338</v>
+        <v>285</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>344</v>
+        <v>292</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>429</v>
+        <v>293</v>
       </c>
       <c r="G49" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H49" s="24" t="s">
-        <v>345</v>
+        <v>294</v>
       </c>
       <c r="I49" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J49" s="23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K49" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L49" s="24"/>
       <c r="M49" s="23" t="s">
-        <v>346</v>
+        <v>295</v>
       </c>
       <c r="N49" s="26"/>
       <c r="O49" s="26"/>
     </row>
     <row r="50" spans="1:15" ht="57" customHeight="1">
       <c r="A50" s="23" t="s">
-        <v>347</v>
+        <v>296</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>348</v>
+        <v>297</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>338</v>
+        <v>285</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>349</v>
+        <v>298</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>430</v>
+        <v>299</v>
       </c>
       <c r="G50" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H50" s="24" t="s">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="I50" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J50" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K50" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L50" s="24"/>
       <c r="M50" s="23" t="s">
-        <v>351</v>
+        <v>301</v>
       </c>
       <c r="N50" s="26"/>
       <c r="O50" s="26"/>
     </row>
     <row r="51" spans="1:15" ht="57" customHeight="1">
       <c r="A51" s="23" t="s">
-        <v>352</v>
+        <v>302</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>287</v>
+        <v>219</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>353</v>
+        <v>303</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>338</v>
+        <v>285</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>354</v>
+        <v>304</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>431</v>
+        <v>305</v>
       </c>
       <c r="G51" s="23" t="s">
         <v>2</v>
       </c>
       <c r="H51" s="24" t="s">
-        <v>355</v>
+        <v>306</v>
       </c>
       <c r="I51" s="23" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="J51" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K51" s="23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L51" s="24"/>
       <c r="M51" s="23" t="s">
-        <v>356</v>
+        <v>307</v>
       </c>
       <c r="N51" s="26"/>
       <c r="O51" s="26"/>
@@ -5019,7 +4890,6 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A4:M5"/>
   </mergeCells>
-  <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="G8:G107">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Fully Covered"/>
     <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Partially Covered"/>
@@ -5066,117 +4936,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1">
-      <c r="A1" s="40" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
+      <c r="A1" s="38" t="s">
+        <v>308</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
     </row>
     <row r="2" spans="1:4" ht="24" customHeight="1">
-      <c r="A2" s="41" t="s">
-        <v>226</v>
-      </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
+      <c r="A2" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
     </row>
     <row r="4" spans="1:4" ht="38" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>227</v>
+        <v>310</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>228</v>
+        <v>311</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>229</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="264.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>230</v>
+        <v>313</v>
       </c>
       <c r="C5" s="5">
         <v>18</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>231</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="264.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>232</v>
+        <v>315</v>
       </c>
       <c r="C6" s="5">
         <v>10</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>233</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="264.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>234</v>
+        <v>317</v>
       </c>
       <c r="C7" s="5">
         <v>8</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>235</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="264.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>236</v>
+        <v>319</v>
       </c>
       <c r="C8" s="5">
         <v>10</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>237</v>
+        <v>320</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="264.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>238</v>
+        <v>321</v>
       </c>
       <c r="C9" s="5">
         <v>8</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>239</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="264.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>240</v>
+        <v>323</v>
       </c>
       <c r="C10" s="5">
         <v>11</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>241</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="264.5" customHeight="1">
@@ -5184,279 +5054,279 @@
         <v>79</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>242</v>
+        <v>325</v>
       </c>
       <c r="C11" s="5">
         <v>5</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>243</v>
+        <v>326</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="264.5" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>244</v>
+        <v>327</v>
       </c>
       <c r="C12" s="5">
         <v>9</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>245</v>
+        <v>328</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="264.5" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>246</v>
+        <v>329</v>
       </c>
       <c r="C13" s="5">
         <v>8</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>247</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="264.5" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>248</v>
+        <v>331</v>
       </c>
       <c r="C14" s="5">
         <v>7</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>249</v>
+        <v>332</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="264.5" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>250</v>
+        <v>333</v>
       </c>
       <c r="C15" s="5">
         <v>8</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>251</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="264.5" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>252</v>
+        <v>335</v>
       </c>
       <c r="C16" s="5">
         <v>10</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>253</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="264.5" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>254</v>
+        <v>337</v>
       </c>
       <c r="C17" s="5">
         <v>9</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>255</v>
+        <v>338</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="264.5" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>256</v>
+        <v>339</v>
       </c>
       <c r="C18" s="5">
         <v>20</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>257</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="264.5" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>258</v>
+        <v>341</v>
       </c>
       <c r="C19" s="5">
         <v>18</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>259</v>
+        <v>342</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="264.5" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>260</v>
+        <v>343</v>
       </c>
       <c r="C20" s="5">
         <v>17</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>261</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="264.5" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>262</v>
+        <v>345</v>
       </c>
       <c r="C21" s="5">
         <v>8</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>263</v>
+        <v>346</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="264.5" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>264</v>
+        <v>347</v>
       </c>
       <c r="C22" s="5">
         <v>8</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>265</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="264.5" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>266</v>
+        <v>349</v>
       </c>
       <c r="C23" s="5">
         <v>8</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>267</v>
+        <v>350</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="264.5" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>268</v>
+        <v>351</v>
       </c>
       <c r="C24" s="5">
         <v>12</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>269</v>
+        <v>352</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="264.5" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>270</v>
+        <v>353</v>
       </c>
       <c r="C25" s="5">
         <v>9</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>271</v>
+        <v>354</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="264.5" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>272</v>
+        <v>355</v>
       </c>
       <c r="C26" s="5">
         <v>7</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>273</v>
+        <v>356</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="264.5" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>274</v>
+        <v>357</v>
       </c>
       <c r="C27" s="5">
         <v>15</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>275</v>
+        <v>358</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="264.5" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>276</v>
+        <v>359</v>
       </c>
       <c r="C28" s="5">
         <v>22</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>277</v>
+        <v>360</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="264.5" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>278</v>
+        <v>361</v>
       </c>
       <c r="C29" s="5">
         <v>7</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>279</v>
+        <v>362</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="264.5" customHeight="1">
       <c r="A30" s="9" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>280</v>
+        <v>363</v>
       </c>
       <c r="C30" s="10">
         <v>7</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>281</v>
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -5487,408 +5357,408 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1">
-      <c r="A1" s="28" t="s">
-        <v>357</v>
-      </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="A1" s="53" t="s">
+        <v>365</v>
+      </c>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1">
-      <c r="A2" s="29" t="s">
-        <v>416</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="A2" s="54" t="s">
+        <v>366</v>
+      </c>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
     </row>
     <row r="4" spans="1:8" ht="42" customHeight="1">
       <c r="A4" s="16" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>227</v>
+        <v>310</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="72" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>288</v>
+        <v>220</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5">
         <v>200</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>369</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="72" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>294</v>
+        <v>228</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5">
         <v>405</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="72" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>300</v>
+        <v>235</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5">
         <v>200</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>376</v>
+        <v>385</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="72" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>305</v>
+        <v>241</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>377</v>
+        <v>386</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5">
         <v>405</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="72" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>309</v>
+        <v>246</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>379</v>
+        <v>388</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>371</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>381</v>
+        <v>390</v>
       </c>
       <c r="F9" s="5">
         <v>200</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="72" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>315</v>
+        <v>253</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>380</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>371</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5">
         <v>400</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>384</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="72" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>317</v>
+        <v>259</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="F11" s="5">
         <v>200</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>388</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="72" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>323</v>
+        <v>266</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>389</v>
+        <v>398</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>390</v>
+        <v>399</v>
       </c>
       <c r="F12" s="5">
         <v>400</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>391</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="72" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>328</v>
+        <v>272</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>392</v>
+        <v>401</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5">
         <v>405</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="72" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>332</v>
+        <v>278</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>394</v>
+        <v>403</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>395</v>
+        <v>404</v>
       </c>
       <c r="F14" s="5">
         <v>404</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>396</v>
+        <v>405</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="72" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>337</v>
+        <v>284</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="F15" s="5">
         <v>201</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="72" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>343</v>
+        <v>291</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>401</v>
+        <v>410</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>393</v>
-      </c>
       <c r="E16" s="5" t="s">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="F16" s="5">
         <v>200</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>403</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>348</v>
+        <v>297</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="F17" s="5">
         <v>200</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="J17" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" customHeight="1">
       <c r="A18" s="5" t="s">
-        <v>353</v>
+        <v>303</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>407</v>
+        <v>417</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="F18" s="5">
         <v>200</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>

</xml_diff>